<commit_message>
Add image galleries and Shopee-style listing editor with import preview
</commit_message>
<xml_diff>
--- a/public/product-import-template.xlsx
+++ b/public/product-import-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import" sheetId="1" r:id="Raec00bf644ed4bc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import" sheetId="1" r:id="R7b8d83da965d49d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -38,8 +38,14 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
   </x:numFmts>
-  <x:fonts count="1">
+  <x:fonts count="2">
     <x:font>
+      <x:sz val="12"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
       <x:sz val="12"/>
       <x:color theme="1"/>
       <x:name val="Calibri"/>
@@ -59,8 +65,9 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1">
+  <x:cellXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -290,6 +297,25 @@
     <x:col min="9" max="9" width="12.83203125" customWidth="1"/>
     <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="20" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="20" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="20" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="20" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="20" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="20" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="20" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="20" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="20" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="20" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="20" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="20" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -326,6 +352,63 @@
       <x:c r="K1" t="str">
         <x:v>是否上架</x:v>
       </x:c>
+      <x:c r="L1" s="1" t="str">
+        <x:v>商品ID</x:v>
+      </x:c>
+      <x:c r="M1" s="1" t="str">
+        <x:v>主商品貨號</x:v>
+      </x:c>
+      <x:c r="N1" s="1" t="str">
+        <x:v>規格名稱 1</x:v>
+      </x:c>
+      <x:c r="O1" s="1" t="str">
+        <x:v>規格選項 1</x:v>
+      </x:c>
+      <x:c r="P1" s="1" t="str">
+        <x:v>規格名稱 2</x:v>
+      </x:c>
+      <x:c r="Q1" s="1" t="str">
+        <x:v>規格選項 2</x:v>
+      </x:c>
+      <x:c r="R1" s="1" t="str">
+        <x:v>商品圖片 1</x:v>
+      </x:c>
+      <x:c r="S1" s="1" t="str">
+        <x:v>商品圖片 2</x:v>
+      </x:c>
+      <x:c r="T1" s="1" t="str">
+        <x:v>商品圖片 3</x:v>
+      </x:c>
+      <x:c r="U1" s="1" t="str">
+        <x:v>商品圖片 4</x:v>
+      </x:c>
+      <x:c r="V1" s="1" t="str">
+        <x:v>商品圖片 5</x:v>
+      </x:c>
+      <x:c r="W1" s="1" t="str">
+        <x:v>商品圖片 6</x:v>
+      </x:c>
+      <x:c r="X1" s="1" t="str">
+        <x:v>商品圖片 7</x:v>
+      </x:c>
+      <x:c r="Y1" s="1" t="str">
+        <x:v>商品圖片 8</x:v>
+      </x:c>
+      <x:c r="Z1" s="1" t="str">
+        <x:v>重量(kg)</x:v>
+      </x:c>
+      <x:c r="AA1" s="1" t="str">
+        <x:v>長度(cm)</x:v>
+      </x:c>
+      <x:c r="AB1" s="1" t="str">
+        <x:v>寬度(cm)</x:v>
+      </x:c>
+      <x:c r="AC1" s="1" t="str">
+        <x:v>高度(cm)</x:v>
+      </x:c>
+      <x:c r="AD1" s="1" t="str">
+        <x:v>備貨天數</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
@@ -357,6 +440,22 @@
       <x:c r="K2" t="str">
         <x:v>是</x:v>
       </x:c>
+      <x:c r="L2" t="str"/>
+      <x:c r="M2" t="str">
+        <x:v>SAMPLE-001</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>顏色</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>白色</x:v>
+      </x:c>
+      <x:c r="P2" t="str">
+        <x:v>尺寸</x:v>
+      </x:c>
+      <x:c r="Q2" t="str">
+        <x:v>24cm</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
@@ -387,6 +486,22 @@
       <x:c r="J3" t="str"/>
       <x:c r="K3" t="str">
         <x:v>是</x:v>
+      </x:c>
+      <x:c r="L3" t="str"/>
+      <x:c r="M3" t="str">
+        <x:v>SAMPLE-002</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>顏色</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>藍色</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>尺寸</x:v>
+      </x:c>
+      <x:c r="Q3" t="str">
+        <x:v>M</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>